<commit_message>
Add daily forward curve generation and print functionality; update simulation to utilize new method
</commit_message>
<xml_diff>
--- a/price_paths_test_n2.xlsx
+++ b/price_paths_test_n2.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\H19790\Documents\PythonProjects\my_project_storage_flex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661BBC40-9D09-4223-B094-9229805F11A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92F6B6FB-8715-491F-BDCF-E00471145F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19860" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{7ECE9F35-DAB4-4C93-B351-872F619E86C7}"/>
   </bookViews>
   <sheets>
     <sheet name="price_paths_test_n2" sheetId="1" r:id="rId1"/>
+    <sheet name="daily_fwd_curve_test" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">daily_fwd_curve_test!$B$1:$D$337</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>-&gt; for i</t>
   </si>
@@ -111,6 +115,15 @@
   </si>
   <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Forward_Price</t>
+  </si>
+  <si>
+    <t>Is_Pillar</t>
   </si>
 </sst>
 </file>
@@ -7091,16 +7104,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>472440</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1013460</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>731520</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7125,6 +7138,67 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>865880</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>99143</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5154C924-2E9F-1D61-32C9-732A67AB1B0C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9133580" y="99060"/>
+          <a:ext cx="3614763" cy="2682240"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -23761,6 +23835,3729 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4DFB22-8CED-4A0D-BA7D-5E036AC4DBFC}">
+  <dimension ref="B1:D337"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B2" s="2">
+        <v>46143</v>
+      </c>
+      <c r="C2">
+        <v>35</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B3" s="2">
+        <v>46144</v>
+      </c>
+      <c r="C3">
+        <v>35</v>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="2">
+        <v>46145</v>
+      </c>
+      <c r="C4">
+        <v>35</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5" s="2">
+        <v>46146</v>
+      </c>
+      <c r="C5">
+        <v>35</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="2">
+        <v>46147</v>
+      </c>
+      <c r="C6">
+        <v>35</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="2">
+        <v>46148</v>
+      </c>
+      <c r="C7">
+        <v>35</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B8" s="2">
+        <v>46149</v>
+      </c>
+      <c r="C8">
+        <v>35</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="2">
+        <v>46150</v>
+      </c>
+      <c r="C9">
+        <v>35</v>
+      </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="2">
+        <v>46151</v>
+      </c>
+      <c r="C10">
+        <v>35</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B11" s="2">
+        <v>46152</v>
+      </c>
+      <c r="C11">
+        <v>35</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B12" s="2">
+        <v>46153</v>
+      </c>
+      <c r="C12">
+        <v>35</v>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B13" s="2">
+        <v>46154</v>
+      </c>
+      <c r="C13">
+        <v>35</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B14" s="2">
+        <v>46155</v>
+      </c>
+      <c r="C14">
+        <v>35</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B15" s="2">
+        <v>46156</v>
+      </c>
+      <c r="C15">
+        <v>35</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B16" s="2">
+        <v>46157</v>
+      </c>
+      <c r="C16">
+        <v>35</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="2">
+        <v>46158</v>
+      </c>
+      <c r="C17">
+        <v>35</v>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="2">
+        <v>46159</v>
+      </c>
+      <c r="C18">
+        <v>35</v>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B19" s="2">
+        <v>46160</v>
+      </c>
+      <c r="C19">
+        <v>35</v>
+      </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="2">
+        <v>46161</v>
+      </c>
+      <c r="C20">
+        <v>35</v>
+      </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="2">
+        <v>46162</v>
+      </c>
+      <c r="C21">
+        <v>35</v>
+      </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="2">
+        <v>46163</v>
+      </c>
+      <c r="C22">
+        <v>35</v>
+      </c>
+      <c r="D22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B23" s="2">
+        <v>46164</v>
+      </c>
+      <c r="C23">
+        <v>35</v>
+      </c>
+      <c r="D23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B24" s="2">
+        <v>46165</v>
+      </c>
+      <c r="C24">
+        <v>35</v>
+      </c>
+      <c r="D24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="2">
+        <v>46166</v>
+      </c>
+      <c r="C25">
+        <v>35</v>
+      </c>
+      <c r="D25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B26" s="2">
+        <v>46167</v>
+      </c>
+      <c r="C26">
+        <v>35</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B27" s="2">
+        <v>46168</v>
+      </c>
+      <c r="C27">
+        <v>35</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B28" s="2">
+        <v>46169</v>
+      </c>
+      <c r="C28">
+        <v>35</v>
+      </c>
+      <c r="D28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="2">
+        <v>46170</v>
+      </c>
+      <c r="C29">
+        <v>35</v>
+      </c>
+      <c r="D29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B30" s="2">
+        <v>46171</v>
+      </c>
+      <c r="C30">
+        <v>35</v>
+      </c>
+      <c r="D30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B31" s="2">
+        <v>46172</v>
+      </c>
+      <c r="C31">
+        <v>35</v>
+      </c>
+      <c r="D31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B32" s="2">
+        <v>46173</v>
+      </c>
+      <c r="C32">
+        <v>35</v>
+      </c>
+      <c r="D32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B33" s="2">
+        <v>46174</v>
+      </c>
+      <c r="C33">
+        <v>35</v>
+      </c>
+      <c r="D33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B34" s="2">
+        <v>46175</v>
+      </c>
+      <c r="C34">
+        <v>35</v>
+      </c>
+      <c r="D34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B35" s="2">
+        <v>46176</v>
+      </c>
+      <c r="C35">
+        <v>35</v>
+      </c>
+      <c r="D35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B36" s="2">
+        <v>46177</v>
+      </c>
+      <c r="C36">
+        <v>35</v>
+      </c>
+      <c r="D36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B37" s="2">
+        <v>46178</v>
+      </c>
+      <c r="C37">
+        <v>35</v>
+      </c>
+      <c r="D37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B38" s="2">
+        <v>46179</v>
+      </c>
+      <c r="C38">
+        <v>35</v>
+      </c>
+      <c r="D38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B39" s="2">
+        <v>46180</v>
+      </c>
+      <c r="C39">
+        <v>35</v>
+      </c>
+      <c r="D39" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B40" s="2">
+        <v>46181</v>
+      </c>
+      <c r="C40">
+        <v>35</v>
+      </c>
+      <c r="D40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B41" s="2">
+        <v>46182</v>
+      </c>
+      <c r="C41">
+        <v>35</v>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B42" s="2">
+        <v>46183</v>
+      </c>
+      <c r="C42">
+        <v>35</v>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B43" s="2">
+        <v>46184</v>
+      </c>
+      <c r="C43">
+        <v>35</v>
+      </c>
+      <c r="D43" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B44" s="2">
+        <v>46185</v>
+      </c>
+      <c r="C44">
+        <v>35</v>
+      </c>
+      <c r="D44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B45" s="2">
+        <v>46186</v>
+      </c>
+      <c r="C45">
+        <v>35</v>
+      </c>
+      <c r="D45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B46" s="2">
+        <v>46187</v>
+      </c>
+      <c r="C46">
+        <v>35</v>
+      </c>
+      <c r="D46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B47" s="2">
+        <v>46188</v>
+      </c>
+      <c r="C47">
+        <v>35</v>
+      </c>
+      <c r="D47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B48" s="2">
+        <v>46189</v>
+      </c>
+      <c r="C48">
+        <v>35</v>
+      </c>
+      <c r="D48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B49" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C49">
+        <v>35</v>
+      </c>
+      <c r="D49" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B50" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C50">
+        <v>35</v>
+      </c>
+      <c r="D50" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B51" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C51">
+        <v>35</v>
+      </c>
+      <c r="D51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B52" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C52">
+        <v>35</v>
+      </c>
+      <c r="D52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B53" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C53">
+        <v>35</v>
+      </c>
+      <c r="D53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B54" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C54">
+        <v>35</v>
+      </c>
+      <c r="D54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B55" s="2">
+        <v>46196</v>
+      </c>
+      <c r="C55">
+        <v>35</v>
+      </c>
+      <c r="D55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B56" s="2">
+        <v>46197</v>
+      </c>
+      <c r="C56">
+        <v>35</v>
+      </c>
+      <c r="D56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B57" s="2">
+        <v>46198</v>
+      </c>
+      <c r="C57">
+        <v>35</v>
+      </c>
+      <c r="D57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B58" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C58">
+        <v>35</v>
+      </c>
+      <c r="D58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B59" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C59">
+        <v>35</v>
+      </c>
+      <c r="D59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B60" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C60">
+        <v>35</v>
+      </c>
+      <c r="D60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B61" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C61">
+        <v>35</v>
+      </c>
+      <c r="D61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B62" s="2">
+        <v>46203</v>
+      </c>
+      <c r="C62">
+        <v>35</v>
+      </c>
+      <c r="D62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B63" s="2">
+        <v>46204</v>
+      </c>
+      <c r="C63">
+        <v>35</v>
+      </c>
+      <c r="D63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B64" s="2">
+        <v>46205</v>
+      </c>
+      <c r="C64">
+        <v>35</v>
+      </c>
+      <c r="D64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B65" s="2">
+        <v>46206</v>
+      </c>
+      <c r="C65">
+        <v>35</v>
+      </c>
+      <c r="D65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B66" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C66">
+        <v>35</v>
+      </c>
+      <c r="D66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B67" s="2">
+        <v>46208</v>
+      </c>
+      <c r="C67">
+        <v>35</v>
+      </c>
+      <c r="D67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B68" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C68">
+        <v>35</v>
+      </c>
+      <c r="D68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B69" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C69">
+        <v>35</v>
+      </c>
+      <c r="D69" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B70" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C70">
+        <v>35</v>
+      </c>
+      <c r="D70" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B71" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C71">
+        <v>35</v>
+      </c>
+      <c r="D71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B72" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C72">
+        <v>35</v>
+      </c>
+      <c r="D72" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B73" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C73">
+        <v>35</v>
+      </c>
+      <c r="D73" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B74" s="2">
+        <v>46215</v>
+      </c>
+      <c r="C74">
+        <v>35</v>
+      </c>
+      <c r="D74" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B75" s="2">
+        <v>46216</v>
+      </c>
+      <c r="C75">
+        <v>35</v>
+      </c>
+      <c r="D75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B76" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C76">
+        <v>35</v>
+      </c>
+      <c r="D76" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B77" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C77">
+        <v>35</v>
+      </c>
+      <c r="D77" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B78" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C78">
+        <v>35</v>
+      </c>
+      <c r="D78" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B79" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C79">
+        <v>35</v>
+      </c>
+      <c r="D79" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B80" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C80">
+        <v>35</v>
+      </c>
+      <c r="D80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B81" s="2">
+        <v>46222</v>
+      </c>
+      <c r="C81">
+        <v>35</v>
+      </c>
+      <c r="D81" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B82" s="2">
+        <v>46223</v>
+      </c>
+      <c r="C82">
+        <v>35</v>
+      </c>
+      <c r="D82" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B83" s="2">
+        <v>46224</v>
+      </c>
+      <c r="C83">
+        <v>35</v>
+      </c>
+      <c r="D83" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B84" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C84">
+        <v>35</v>
+      </c>
+      <c r="D84" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B85" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C85">
+        <v>35</v>
+      </c>
+      <c r="D85" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B86" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C86">
+        <v>35</v>
+      </c>
+      <c r="D86" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B87" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C87">
+        <v>35</v>
+      </c>
+      <c r="D87" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B88" s="2">
+        <v>46229</v>
+      </c>
+      <c r="C88">
+        <v>35</v>
+      </c>
+      <c r="D88" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B89" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C89">
+        <v>35</v>
+      </c>
+      <c r="D89" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B90" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C90">
+        <v>35</v>
+      </c>
+      <c r="D90" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B91" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C91">
+        <v>35</v>
+      </c>
+      <c r="D91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B92" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C92">
+        <v>35</v>
+      </c>
+      <c r="D92" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B93" s="2">
+        <v>46234</v>
+      </c>
+      <c r="C93">
+        <v>35</v>
+      </c>
+      <c r="D93" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B94" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C94">
+        <v>35</v>
+      </c>
+      <c r="D94" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B95" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C95">
+        <v>35</v>
+      </c>
+      <c r="D95" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B96" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C96">
+        <v>35</v>
+      </c>
+      <c r="D96" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B97" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C97">
+        <v>35</v>
+      </c>
+      <c r="D97" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B98" s="2">
+        <v>46239</v>
+      </c>
+      <c r="C98">
+        <v>35</v>
+      </c>
+      <c r="D98" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B99" s="2">
+        <v>46240</v>
+      </c>
+      <c r="C99">
+        <v>35</v>
+      </c>
+      <c r="D99" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B100" s="2">
+        <v>46241</v>
+      </c>
+      <c r="C100">
+        <v>35</v>
+      </c>
+      <c r="D100" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B101" s="2">
+        <v>46242</v>
+      </c>
+      <c r="C101">
+        <v>35</v>
+      </c>
+      <c r="D101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B102" s="2">
+        <v>46243</v>
+      </c>
+      <c r="C102">
+        <v>35</v>
+      </c>
+      <c r="D102" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B103" s="2">
+        <v>46244</v>
+      </c>
+      <c r="C103">
+        <v>35</v>
+      </c>
+      <c r="D103" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B104" s="2">
+        <v>46245</v>
+      </c>
+      <c r="C104">
+        <v>35</v>
+      </c>
+      <c r="D104" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B105" s="2">
+        <v>46246</v>
+      </c>
+      <c r="C105">
+        <v>35</v>
+      </c>
+      <c r="D105" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B106" s="2">
+        <v>46247</v>
+      </c>
+      <c r="C106">
+        <v>35</v>
+      </c>
+      <c r="D106" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B107" s="2">
+        <v>46248</v>
+      </c>
+      <c r="C107">
+        <v>35</v>
+      </c>
+      <c r="D107" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B108" s="2">
+        <v>46249</v>
+      </c>
+      <c r="C108">
+        <v>35</v>
+      </c>
+      <c r="D108" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B109" s="2">
+        <v>46250</v>
+      </c>
+      <c r="C109">
+        <v>35</v>
+      </c>
+      <c r="D109" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B110" s="2">
+        <v>46251</v>
+      </c>
+      <c r="C110">
+        <v>35</v>
+      </c>
+      <c r="D110" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B111" s="2">
+        <v>46252</v>
+      </c>
+      <c r="C111">
+        <v>35</v>
+      </c>
+      <c r="D111" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B112" s="2">
+        <v>46253</v>
+      </c>
+      <c r="C112">
+        <v>35</v>
+      </c>
+      <c r="D112" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B113" s="2">
+        <v>46254</v>
+      </c>
+      <c r="C113">
+        <v>35</v>
+      </c>
+      <c r="D113" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B114" s="2">
+        <v>46255</v>
+      </c>
+      <c r="C114">
+        <v>35</v>
+      </c>
+      <c r="D114" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B115" s="2">
+        <v>46256</v>
+      </c>
+      <c r="C115">
+        <v>35</v>
+      </c>
+      <c r="D115" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B116" s="2">
+        <v>46257</v>
+      </c>
+      <c r="C116">
+        <v>35</v>
+      </c>
+      <c r="D116" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B117" s="2">
+        <v>46258</v>
+      </c>
+      <c r="C117">
+        <v>35</v>
+      </c>
+      <c r="D117" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B118" s="2">
+        <v>46259</v>
+      </c>
+      <c r="C118">
+        <v>35</v>
+      </c>
+      <c r="D118" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B119" s="2">
+        <v>46260</v>
+      </c>
+      <c r="C119">
+        <v>35</v>
+      </c>
+      <c r="D119" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B120" s="2">
+        <v>46261</v>
+      </c>
+      <c r="C120">
+        <v>35</v>
+      </c>
+      <c r="D120" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B121" s="2">
+        <v>46262</v>
+      </c>
+      <c r="C121">
+        <v>35</v>
+      </c>
+      <c r="D121" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B122" s="2">
+        <v>46263</v>
+      </c>
+      <c r="C122">
+        <v>35</v>
+      </c>
+      <c r="D122" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B123" s="2">
+        <v>46264</v>
+      </c>
+      <c r="C123">
+        <v>35</v>
+      </c>
+      <c r="D123" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B124" s="2">
+        <v>46265</v>
+      </c>
+      <c r="C124">
+        <v>35</v>
+      </c>
+      <c r="D124" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B125" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C125">
+        <v>35</v>
+      </c>
+      <c r="D125" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B126" s="2">
+        <v>46267</v>
+      </c>
+      <c r="C126">
+        <v>35.166699999999999</v>
+      </c>
+      <c r="D126" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B127" s="2">
+        <v>46268</v>
+      </c>
+      <c r="C127">
+        <v>35.333300000000001</v>
+      </c>
+      <c r="D127" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B128" s="2">
+        <v>46269</v>
+      </c>
+      <c r="C128">
+        <v>35.5</v>
+      </c>
+      <c r="D128" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B129" s="2">
+        <v>46270</v>
+      </c>
+      <c r="C129">
+        <v>35.666699999999999</v>
+      </c>
+      <c r="D129" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B130" s="2">
+        <v>46271</v>
+      </c>
+      <c r="C130">
+        <v>35.833300000000001</v>
+      </c>
+      <c r="D130" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B131" s="2">
+        <v>46272</v>
+      </c>
+      <c r="C131">
+        <v>36</v>
+      </c>
+      <c r="D131" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B132" s="2">
+        <v>46273</v>
+      </c>
+      <c r="C132">
+        <v>36.166699999999999</v>
+      </c>
+      <c r="D132" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B133" s="2">
+        <v>46274</v>
+      </c>
+      <c r="C133">
+        <v>36.333300000000001</v>
+      </c>
+      <c r="D133" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B134" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C134">
+        <v>36.5</v>
+      </c>
+      <c r="D134" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B135" s="2">
+        <v>46276</v>
+      </c>
+      <c r="C135">
+        <v>36.666699999999999</v>
+      </c>
+      <c r="D135" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B136" s="2">
+        <v>46277</v>
+      </c>
+      <c r="C136">
+        <v>36.833300000000001</v>
+      </c>
+      <c r="D136" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B137" s="2">
+        <v>46278</v>
+      </c>
+      <c r="C137">
+        <v>37</v>
+      </c>
+      <c r="D137" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B138" s="2">
+        <v>46279</v>
+      </c>
+      <c r="C138">
+        <v>37.166699999999999</v>
+      </c>
+      <c r="D138" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B139" s="2">
+        <v>46280</v>
+      </c>
+      <c r="C139">
+        <v>37.333300000000001</v>
+      </c>
+      <c r="D139" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B140" s="2">
+        <v>46281</v>
+      </c>
+      <c r="C140">
+        <v>37.5</v>
+      </c>
+      <c r="D140" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B141" s="2">
+        <v>46282</v>
+      </c>
+      <c r="C141">
+        <v>37.666699999999999</v>
+      </c>
+      <c r="D141" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B142" s="2">
+        <v>46283</v>
+      </c>
+      <c r="C142">
+        <v>37.833300000000001</v>
+      </c>
+      <c r="D142" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B143" s="2">
+        <v>46284</v>
+      </c>
+      <c r="C143">
+        <v>38</v>
+      </c>
+      <c r="D143" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B144" s="2">
+        <v>46285</v>
+      </c>
+      <c r="C144">
+        <v>38.166699999999999</v>
+      </c>
+      <c r="D144" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B145" s="2">
+        <v>46286</v>
+      </c>
+      <c r="C145">
+        <v>38.333300000000001</v>
+      </c>
+      <c r="D145" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B146" s="2">
+        <v>46287</v>
+      </c>
+      <c r="C146">
+        <v>38.5</v>
+      </c>
+      <c r="D146" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B147" s="2">
+        <v>46288</v>
+      </c>
+      <c r="C147">
+        <v>38.666699999999999</v>
+      </c>
+      <c r="D147" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B148" s="2">
+        <v>46289</v>
+      </c>
+      <c r="C148">
+        <v>38.833300000000001</v>
+      </c>
+      <c r="D148" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B149" s="2">
+        <v>46290</v>
+      </c>
+      <c r="C149">
+        <v>39</v>
+      </c>
+      <c r="D149" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B150" s="2">
+        <v>46291</v>
+      </c>
+      <c r="C150">
+        <v>39.166699999999999</v>
+      </c>
+      <c r="D150" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B151" s="2">
+        <v>46292</v>
+      </c>
+      <c r="C151">
+        <v>39.333300000000001</v>
+      </c>
+      <c r="D151" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B152" s="2">
+        <v>46293</v>
+      </c>
+      <c r="C152">
+        <v>39.5</v>
+      </c>
+      <c r="D152" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B153" s="2">
+        <v>46294</v>
+      </c>
+      <c r="C153">
+        <v>39.666699999999999</v>
+      </c>
+      <c r="D153" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B154" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C154">
+        <v>39.833300000000001</v>
+      </c>
+      <c r="D154" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B155" s="2">
+        <v>46296</v>
+      </c>
+      <c r="C155">
+        <v>40</v>
+      </c>
+      <c r="D155" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B156" s="2">
+        <v>46297</v>
+      </c>
+      <c r="C156">
+        <v>40</v>
+      </c>
+      <c r="D156" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B157" s="2">
+        <v>46298</v>
+      </c>
+      <c r="C157">
+        <v>40</v>
+      </c>
+      <c r="D157" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B158" s="2">
+        <v>46299</v>
+      </c>
+      <c r="C158">
+        <v>40</v>
+      </c>
+      <c r="D158" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B159" s="2">
+        <v>46300</v>
+      </c>
+      <c r="C159">
+        <v>40</v>
+      </c>
+      <c r="D159" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B160" s="2">
+        <v>46301</v>
+      </c>
+      <c r="C160">
+        <v>40</v>
+      </c>
+      <c r="D160" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B161" s="2">
+        <v>46302</v>
+      </c>
+      <c r="C161">
+        <v>40</v>
+      </c>
+      <c r="D161" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B162" s="2">
+        <v>46303</v>
+      </c>
+      <c r="C162">
+        <v>40</v>
+      </c>
+      <c r="D162" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B163" s="2">
+        <v>46304</v>
+      </c>
+      <c r="C163">
+        <v>40</v>
+      </c>
+      <c r="D163" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B164" s="2">
+        <v>46305</v>
+      </c>
+      <c r="C164">
+        <v>40</v>
+      </c>
+      <c r="D164" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B165" s="2">
+        <v>46306</v>
+      </c>
+      <c r="C165">
+        <v>40</v>
+      </c>
+      <c r="D165" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B166" s="2">
+        <v>46307</v>
+      </c>
+      <c r="C166">
+        <v>40</v>
+      </c>
+      <c r="D166" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B167" s="2">
+        <v>46308</v>
+      </c>
+      <c r="C167">
+        <v>40</v>
+      </c>
+      <c r="D167" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B168" s="2">
+        <v>46309</v>
+      </c>
+      <c r="C168">
+        <v>40</v>
+      </c>
+      <c r="D168" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B169" s="2">
+        <v>46310</v>
+      </c>
+      <c r="C169">
+        <v>40</v>
+      </c>
+      <c r="D169" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B170" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C170">
+        <v>40</v>
+      </c>
+      <c r="D170" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B171" s="2">
+        <v>46312</v>
+      </c>
+      <c r="C171">
+        <v>40</v>
+      </c>
+      <c r="D171" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B172" s="2">
+        <v>46313</v>
+      </c>
+      <c r="C172">
+        <v>40</v>
+      </c>
+      <c r="D172" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B173" s="2">
+        <v>46314</v>
+      </c>
+      <c r="C173">
+        <v>40</v>
+      </c>
+      <c r="D173" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B174" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C174">
+        <v>40</v>
+      </c>
+      <c r="D174" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B175" s="2">
+        <v>46316</v>
+      </c>
+      <c r="C175">
+        <v>40</v>
+      </c>
+      <c r="D175" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B176" s="2">
+        <v>46317</v>
+      </c>
+      <c r="C176">
+        <v>40</v>
+      </c>
+      <c r="D176" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B177" s="2">
+        <v>46318</v>
+      </c>
+      <c r="C177">
+        <v>40</v>
+      </c>
+      <c r="D177" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B178" s="2">
+        <v>46319</v>
+      </c>
+      <c r="C178">
+        <v>40</v>
+      </c>
+      <c r="D178" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B179" s="2">
+        <v>46320</v>
+      </c>
+      <c r="C179">
+        <v>40</v>
+      </c>
+      <c r="D179" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B180" s="2">
+        <v>46321</v>
+      </c>
+      <c r="C180">
+        <v>40</v>
+      </c>
+      <c r="D180" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B181" s="2">
+        <v>46322</v>
+      </c>
+      <c r="C181">
+        <v>40</v>
+      </c>
+      <c r="D181" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B182" s="2">
+        <v>46323</v>
+      </c>
+      <c r="C182">
+        <v>40</v>
+      </c>
+      <c r="D182" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B183" s="2">
+        <v>46324</v>
+      </c>
+      <c r="C183">
+        <v>40</v>
+      </c>
+      <c r="D183" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B184" s="2">
+        <v>46325</v>
+      </c>
+      <c r="C184">
+        <v>40</v>
+      </c>
+      <c r="D184" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B185" s="2">
+        <v>46326</v>
+      </c>
+      <c r="C185">
+        <v>40</v>
+      </c>
+      <c r="D185" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B186" s="2">
+        <v>46327</v>
+      </c>
+      <c r="C186">
+        <v>40</v>
+      </c>
+      <c r="D186" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B187" s="2">
+        <v>46328</v>
+      </c>
+      <c r="C187">
+        <v>40</v>
+      </c>
+      <c r="D187" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B188" s="2">
+        <v>46329</v>
+      </c>
+      <c r="C188">
+        <v>40</v>
+      </c>
+      <c r="D188" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B189" s="2">
+        <v>46330</v>
+      </c>
+      <c r="C189">
+        <v>40</v>
+      </c>
+      <c r="D189" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B190" s="2">
+        <v>46331</v>
+      </c>
+      <c r="C190">
+        <v>40</v>
+      </c>
+      <c r="D190" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B191" s="2">
+        <v>46332</v>
+      </c>
+      <c r="C191">
+        <v>40</v>
+      </c>
+      <c r="D191" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B192" s="2">
+        <v>46333</v>
+      </c>
+      <c r="C192">
+        <v>40</v>
+      </c>
+      <c r="D192" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B193" s="2">
+        <v>46334</v>
+      </c>
+      <c r="C193">
+        <v>40</v>
+      </c>
+      <c r="D193" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B194" s="2">
+        <v>46335</v>
+      </c>
+      <c r="C194">
+        <v>40</v>
+      </c>
+      <c r="D194" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B195" s="2">
+        <v>46336</v>
+      </c>
+      <c r="C195">
+        <v>40</v>
+      </c>
+      <c r="D195" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B196" s="2">
+        <v>46337</v>
+      </c>
+      <c r="C196">
+        <v>40</v>
+      </c>
+      <c r="D196" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B197" s="2">
+        <v>46338</v>
+      </c>
+      <c r="C197">
+        <v>40</v>
+      </c>
+      <c r="D197" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B198" s="2">
+        <v>46339</v>
+      </c>
+      <c r="C198">
+        <v>40</v>
+      </c>
+      <c r="D198" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B199" s="2">
+        <v>46340</v>
+      </c>
+      <c r="C199">
+        <v>40</v>
+      </c>
+      <c r="D199" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B200" s="2">
+        <v>46341</v>
+      </c>
+      <c r="C200">
+        <v>40</v>
+      </c>
+      <c r="D200" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B201" s="2">
+        <v>46342</v>
+      </c>
+      <c r="C201">
+        <v>40</v>
+      </c>
+      <c r="D201" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B202" s="2">
+        <v>46343</v>
+      </c>
+      <c r="C202">
+        <v>40</v>
+      </c>
+      <c r="D202" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B203" s="2">
+        <v>46344</v>
+      </c>
+      <c r="C203">
+        <v>40</v>
+      </c>
+      <c r="D203" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B204" s="2">
+        <v>46345</v>
+      </c>
+      <c r="C204">
+        <v>40</v>
+      </c>
+      <c r="D204" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B205" s="2">
+        <v>46346</v>
+      </c>
+      <c r="C205">
+        <v>40</v>
+      </c>
+      <c r="D205" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B206" s="2">
+        <v>46347</v>
+      </c>
+      <c r="C206">
+        <v>40</v>
+      </c>
+      <c r="D206" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B207" s="2">
+        <v>46348</v>
+      </c>
+      <c r="C207">
+        <v>40</v>
+      </c>
+      <c r="D207" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B208" s="2">
+        <v>46349</v>
+      </c>
+      <c r="C208">
+        <v>40</v>
+      </c>
+      <c r="D208" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B209" s="2">
+        <v>46350</v>
+      </c>
+      <c r="C209">
+        <v>40</v>
+      </c>
+      <c r="D209" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B210" s="2">
+        <v>46351</v>
+      </c>
+      <c r="C210">
+        <v>40</v>
+      </c>
+      <c r="D210" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B211" s="2">
+        <v>46352</v>
+      </c>
+      <c r="C211">
+        <v>40</v>
+      </c>
+      <c r="D211" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B212" s="2">
+        <v>46353</v>
+      </c>
+      <c r="C212">
+        <v>40</v>
+      </c>
+      <c r="D212" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B213" s="2">
+        <v>46354</v>
+      </c>
+      <c r="C213">
+        <v>40</v>
+      </c>
+      <c r="D213" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B214" s="2">
+        <v>46355</v>
+      </c>
+      <c r="C214">
+        <v>40</v>
+      </c>
+      <c r="D214" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B215" s="2">
+        <v>46356</v>
+      </c>
+      <c r="C215">
+        <v>40</v>
+      </c>
+      <c r="D215" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B216" s="2">
+        <v>46357</v>
+      </c>
+      <c r="C216">
+        <v>40</v>
+      </c>
+      <c r="D216" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B217" s="2">
+        <v>46358</v>
+      </c>
+      <c r="C217">
+        <v>40</v>
+      </c>
+      <c r="D217" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B218" s="2">
+        <v>46359</v>
+      </c>
+      <c r="C218">
+        <v>40</v>
+      </c>
+      <c r="D218" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B219" s="2">
+        <v>46360</v>
+      </c>
+      <c r="C219">
+        <v>40</v>
+      </c>
+      <c r="D219" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B220" s="2">
+        <v>46361</v>
+      </c>
+      <c r="C220">
+        <v>40</v>
+      </c>
+      <c r="D220" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B221" s="2">
+        <v>46362</v>
+      </c>
+      <c r="C221">
+        <v>40</v>
+      </c>
+      <c r="D221" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B222" s="2">
+        <v>46363</v>
+      </c>
+      <c r="C222">
+        <v>40</v>
+      </c>
+      <c r="D222" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B223" s="2">
+        <v>46364</v>
+      </c>
+      <c r="C223">
+        <v>40</v>
+      </c>
+      <c r="D223" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B224" s="2">
+        <v>46365</v>
+      </c>
+      <c r="C224">
+        <v>40</v>
+      </c>
+      <c r="D224" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B225" s="2">
+        <v>46366</v>
+      </c>
+      <c r="C225">
+        <v>40</v>
+      </c>
+      <c r="D225" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B226" s="2">
+        <v>46367</v>
+      </c>
+      <c r="C226">
+        <v>40</v>
+      </c>
+      <c r="D226" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B227" s="2">
+        <v>46368</v>
+      </c>
+      <c r="C227">
+        <v>40</v>
+      </c>
+      <c r="D227" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B228" s="2">
+        <v>46369</v>
+      </c>
+      <c r="C228">
+        <v>40</v>
+      </c>
+      <c r="D228" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B229" s="2">
+        <v>46370</v>
+      </c>
+      <c r="C229">
+        <v>40</v>
+      </c>
+      <c r="D229" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B230" s="2">
+        <v>46371</v>
+      </c>
+      <c r="C230">
+        <v>40</v>
+      </c>
+      <c r="D230" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B231" s="2">
+        <v>46372</v>
+      </c>
+      <c r="C231">
+        <v>40</v>
+      </c>
+      <c r="D231" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B232" s="2">
+        <v>46373</v>
+      </c>
+      <c r="C232">
+        <v>40</v>
+      </c>
+      <c r="D232" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B233" s="2">
+        <v>46374</v>
+      </c>
+      <c r="C233">
+        <v>40</v>
+      </c>
+      <c r="D233" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B234" s="2">
+        <v>46375</v>
+      </c>
+      <c r="C234">
+        <v>40</v>
+      </c>
+      <c r="D234" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B235" s="2">
+        <v>46376</v>
+      </c>
+      <c r="C235">
+        <v>40</v>
+      </c>
+      <c r="D235" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B236" s="2">
+        <v>46377</v>
+      </c>
+      <c r="C236">
+        <v>40</v>
+      </c>
+      <c r="D236" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B237" s="2">
+        <v>46378</v>
+      </c>
+      <c r="C237">
+        <v>40</v>
+      </c>
+      <c r="D237" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B238" s="2">
+        <v>46379</v>
+      </c>
+      <c r="C238">
+        <v>40</v>
+      </c>
+      <c r="D238" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B239" s="2">
+        <v>46380</v>
+      </c>
+      <c r="C239">
+        <v>40</v>
+      </c>
+      <c r="D239" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B240" s="2">
+        <v>46381</v>
+      </c>
+      <c r="C240">
+        <v>40</v>
+      </c>
+      <c r="D240" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B241" s="2">
+        <v>46382</v>
+      </c>
+      <c r="C241">
+        <v>40</v>
+      </c>
+      <c r="D241" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B242" s="2">
+        <v>46383</v>
+      </c>
+      <c r="C242">
+        <v>40</v>
+      </c>
+      <c r="D242" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B243" s="2">
+        <v>46384</v>
+      </c>
+      <c r="C243">
+        <v>40</v>
+      </c>
+      <c r="D243" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B244" s="2">
+        <v>46385</v>
+      </c>
+      <c r="C244">
+        <v>40</v>
+      </c>
+      <c r="D244" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B245" s="2">
+        <v>46386</v>
+      </c>
+      <c r="C245">
+        <v>40</v>
+      </c>
+      <c r="D245" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B246" s="2">
+        <v>46387</v>
+      </c>
+      <c r="C246">
+        <v>40</v>
+      </c>
+      <c r="D246" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B247" s="2">
+        <v>46388</v>
+      </c>
+      <c r="C247">
+        <v>40</v>
+      </c>
+      <c r="D247" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B248" s="2">
+        <v>46389</v>
+      </c>
+      <c r="C248">
+        <v>40</v>
+      </c>
+      <c r="D248" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B249" s="2">
+        <v>46390</v>
+      </c>
+      <c r="C249">
+        <v>40</v>
+      </c>
+      <c r="D249" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B250" s="2">
+        <v>46391</v>
+      </c>
+      <c r="C250">
+        <v>40</v>
+      </c>
+      <c r="D250" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B251" s="2">
+        <v>46392</v>
+      </c>
+      <c r="C251">
+        <v>40</v>
+      </c>
+      <c r="D251" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B252" s="2">
+        <v>46393</v>
+      </c>
+      <c r="C252">
+        <v>40</v>
+      </c>
+      <c r="D252" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B253" s="2">
+        <v>46394</v>
+      </c>
+      <c r="C253">
+        <v>40</v>
+      </c>
+      <c r="D253" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B254" s="2">
+        <v>46395</v>
+      </c>
+      <c r="C254">
+        <v>40</v>
+      </c>
+      <c r="D254" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="255" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B255" s="2">
+        <v>46396</v>
+      </c>
+      <c r="C255">
+        <v>40</v>
+      </c>
+      <c r="D255" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="256" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B256" s="2">
+        <v>46397</v>
+      </c>
+      <c r="C256">
+        <v>40</v>
+      </c>
+      <c r="D256" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B257" s="2">
+        <v>46398</v>
+      </c>
+      <c r="C257">
+        <v>40</v>
+      </c>
+      <c r="D257" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B258" s="2">
+        <v>46399</v>
+      </c>
+      <c r="C258">
+        <v>40</v>
+      </c>
+      <c r="D258" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B259" s="2">
+        <v>46400</v>
+      </c>
+      <c r="C259">
+        <v>40</v>
+      </c>
+      <c r="D259" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B260" s="2">
+        <v>46401</v>
+      </c>
+      <c r="C260">
+        <v>40</v>
+      </c>
+      <c r="D260" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B261" s="2">
+        <v>46402</v>
+      </c>
+      <c r="C261">
+        <v>40</v>
+      </c>
+      <c r="D261" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B262" s="2">
+        <v>46403</v>
+      </c>
+      <c r="C262">
+        <v>40</v>
+      </c>
+      <c r="D262" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B263" s="2">
+        <v>46404</v>
+      </c>
+      <c r="C263">
+        <v>40</v>
+      </c>
+      <c r="D263" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B264" s="2">
+        <v>46405</v>
+      </c>
+      <c r="C264">
+        <v>40</v>
+      </c>
+      <c r="D264" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B265" s="2">
+        <v>46406</v>
+      </c>
+      <c r="C265">
+        <v>40</v>
+      </c>
+      <c r="D265" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B266" s="2">
+        <v>46407</v>
+      </c>
+      <c r="C266">
+        <v>40</v>
+      </c>
+      <c r="D266" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B267" s="2">
+        <v>46408</v>
+      </c>
+      <c r="C267">
+        <v>40</v>
+      </c>
+      <c r="D267" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B268" s="2">
+        <v>46409</v>
+      </c>
+      <c r="C268">
+        <v>40</v>
+      </c>
+      <c r="D268" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B269" s="2">
+        <v>46410</v>
+      </c>
+      <c r="C269">
+        <v>40</v>
+      </c>
+      <c r="D269" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B270" s="2">
+        <v>46411</v>
+      </c>
+      <c r="C270">
+        <v>40</v>
+      </c>
+      <c r="D270" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B271" s="2">
+        <v>46412</v>
+      </c>
+      <c r="C271">
+        <v>40</v>
+      </c>
+      <c r="D271" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B272" s="2">
+        <v>46413</v>
+      </c>
+      <c r="C272">
+        <v>40</v>
+      </c>
+      <c r="D272" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B273" s="2">
+        <v>46414</v>
+      </c>
+      <c r="C273">
+        <v>40</v>
+      </c>
+      <c r="D273" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B274" s="2">
+        <v>46415</v>
+      </c>
+      <c r="C274">
+        <v>40</v>
+      </c>
+      <c r="D274" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B275" s="2">
+        <v>46416</v>
+      </c>
+      <c r="C275">
+        <v>40</v>
+      </c>
+      <c r="D275" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B276" s="2">
+        <v>46417</v>
+      </c>
+      <c r="C276">
+        <v>40</v>
+      </c>
+      <c r="D276" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B277" s="2">
+        <v>46418</v>
+      </c>
+      <c r="C277">
+        <v>40</v>
+      </c>
+      <c r="D277" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B278" s="2">
+        <v>46419</v>
+      </c>
+      <c r="C278">
+        <v>40</v>
+      </c>
+      <c r="D278" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="279" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B279" s="2">
+        <v>46420</v>
+      </c>
+      <c r="C279">
+        <v>40</v>
+      </c>
+      <c r="D279" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B280" s="2">
+        <v>46421</v>
+      </c>
+      <c r="C280">
+        <v>40</v>
+      </c>
+      <c r="D280" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B281" s="2">
+        <v>46422</v>
+      </c>
+      <c r="C281">
+        <v>40</v>
+      </c>
+      <c r="D281" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B282" s="2">
+        <v>46423</v>
+      </c>
+      <c r="C282">
+        <v>40</v>
+      </c>
+      <c r="D282" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B283" s="2">
+        <v>46424</v>
+      </c>
+      <c r="C283">
+        <v>40</v>
+      </c>
+      <c r="D283" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B284" s="2">
+        <v>46425</v>
+      </c>
+      <c r="C284">
+        <v>40</v>
+      </c>
+      <c r="D284" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B285" s="2">
+        <v>46426</v>
+      </c>
+      <c r="C285">
+        <v>40</v>
+      </c>
+      <c r="D285" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="286" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B286" s="2">
+        <v>46427</v>
+      </c>
+      <c r="C286">
+        <v>40</v>
+      </c>
+      <c r="D286" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B287" s="2">
+        <v>46428</v>
+      </c>
+      <c r="C287">
+        <v>40</v>
+      </c>
+      <c r="D287" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B288" s="2">
+        <v>46429</v>
+      </c>
+      <c r="C288">
+        <v>40</v>
+      </c>
+      <c r="D288" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B289" s="2">
+        <v>46430</v>
+      </c>
+      <c r="C289">
+        <v>40</v>
+      </c>
+      <c r="D289" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B290" s="2">
+        <v>46431</v>
+      </c>
+      <c r="C290">
+        <v>40</v>
+      </c>
+      <c r="D290" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B291" s="2">
+        <v>46432</v>
+      </c>
+      <c r="C291">
+        <v>40</v>
+      </c>
+      <c r="D291" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B292" s="2">
+        <v>46433</v>
+      </c>
+      <c r="C292">
+        <v>40</v>
+      </c>
+      <c r="D292" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B293" s="2">
+        <v>46434</v>
+      </c>
+      <c r="C293">
+        <v>40</v>
+      </c>
+      <c r="D293" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B294" s="2">
+        <v>46435</v>
+      </c>
+      <c r="C294">
+        <v>40</v>
+      </c>
+      <c r="D294" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B295" s="2">
+        <v>46436</v>
+      </c>
+      <c r="C295">
+        <v>40</v>
+      </c>
+      <c r="D295" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B296" s="2">
+        <v>46437</v>
+      </c>
+      <c r="C296">
+        <v>40</v>
+      </c>
+      <c r="D296" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B297" s="2">
+        <v>46438</v>
+      </c>
+      <c r="C297">
+        <v>40</v>
+      </c>
+      <c r="D297" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B298" s="2">
+        <v>46439</v>
+      </c>
+      <c r="C298">
+        <v>40</v>
+      </c>
+      <c r="D298" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B299" s="2">
+        <v>46440</v>
+      </c>
+      <c r="C299">
+        <v>40</v>
+      </c>
+      <c r="D299" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B300" s="2">
+        <v>46441</v>
+      </c>
+      <c r="C300">
+        <v>40</v>
+      </c>
+      <c r="D300" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B301" s="2">
+        <v>46442</v>
+      </c>
+      <c r="C301">
+        <v>40</v>
+      </c>
+      <c r="D301" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B302" s="2">
+        <v>46443</v>
+      </c>
+      <c r="C302">
+        <v>40</v>
+      </c>
+      <c r="D302" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B303" s="2">
+        <v>46444</v>
+      </c>
+      <c r="C303">
+        <v>40</v>
+      </c>
+      <c r="D303" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B304" s="2">
+        <v>46445</v>
+      </c>
+      <c r="C304">
+        <v>40</v>
+      </c>
+      <c r="D304" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B305" s="2">
+        <v>46446</v>
+      </c>
+      <c r="C305">
+        <v>40</v>
+      </c>
+      <c r="D305" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B306" s="2">
+        <v>46447</v>
+      </c>
+      <c r="C306">
+        <v>40</v>
+      </c>
+      <c r="D306" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="307" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B307" s="2">
+        <v>46448</v>
+      </c>
+      <c r="C307">
+        <v>40</v>
+      </c>
+      <c r="D307" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B308" s="2">
+        <v>46449</v>
+      </c>
+      <c r="C308">
+        <v>40</v>
+      </c>
+      <c r="D308" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B309" s="2">
+        <v>46450</v>
+      </c>
+      <c r="C309">
+        <v>40</v>
+      </c>
+      <c r="D309" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B310" s="2">
+        <v>46451</v>
+      </c>
+      <c r="C310">
+        <v>40</v>
+      </c>
+      <c r="D310" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B311" s="2">
+        <v>46452</v>
+      </c>
+      <c r="C311">
+        <v>40</v>
+      </c>
+      <c r="D311" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B312" s="2">
+        <v>46453</v>
+      </c>
+      <c r="C312">
+        <v>40</v>
+      </c>
+      <c r="D312" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B313" s="2">
+        <v>46454</v>
+      </c>
+      <c r="C313">
+        <v>40</v>
+      </c>
+      <c r="D313" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B314" s="2">
+        <v>46455</v>
+      </c>
+      <c r="C314">
+        <v>40</v>
+      </c>
+      <c r="D314" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B315" s="2">
+        <v>46456</v>
+      </c>
+      <c r="C315">
+        <v>40</v>
+      </c>
+      <c r="D315" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B316" s="2">
+        <v>46457</v>
+      </c>
+      <c r="C316">
+        <v>40</v>
+      </c>
+      <c r="D316" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B317" s="2">
+        <v>46458</v>
+      </c>
+      <c r="C317">
+        <v>40</v>
+      </c>
+      <c r="D317" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B318" s="2">
+        <v>46459</v>
+      </c>
+      <c r="C318">
+        <v>40</v>
+      </c>
+      <c r="D318" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B319" s="2">
+        <v>46460</v>
+      </c>
+      <c r="C319">
+        <v>40</v>
+      </c>
+      <c r="D319" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B320" s="2">
+        <v>46461</v>
+      </c>
+      <c r="C320">
+        <v>40</v>
+      </c>
+      <c r="D320" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B321" s="2">
+        <v>46462</v>
+      </c>
+      <c r="C321">
+        <v>40</v>
+      </c>
+      <c r="D321" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B322" s="2">
+        <v>46463</v>
+      </c>
+      <c r="C322">
+        <v>40</v>
+      </c>
+      <c r="D322" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B323" s="2">
+        <v>46464</v>
+      </c>
+      <c r="C323">
+        <v>40</v>
+      </c>
+      <c r="D323" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B324" s="2">
+        <v>46465</v>
+      </c>
+      <c r="C324">
+        <v>40</v>
+      </c>
+      <c r="D324" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B325" s="2">
+        <v>46466</v>
+      </c>
+      <c r="C325">
+        <v>40</v>
+      </c>
+      <c r="D325" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B326" s="2">
+        <v>46467</v>
+      </c>
+      <c r="C326">
+        <v>40</v>
+      </c>
+      <c r="D326" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B327" s="2">
+        <v>46468</v>
+      </c>
+      <c r="C327">
+        <v>40</v>
+      </c>
+      <c r="D327" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B328" s="2">
+        <v>46469</v>
+      </c>
+      <c r="C328">
+        <v>40</v>
+      </c>
+      <c r="D328" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B329" s="2">
+        <v>46470</v>
+      </c>
+      <c r="C329">
+        <v>40</v>
+      </c>
+      <c r="D329" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B330" s="2">
+        <v>46471</v>
+      </c>
+      <c r="C330">
+        <v>40</v>
+      </c>
+      <c r="D330" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B331" s="2">
+        <v>46472</v>
+      </c>
+      <c r="C331">
+        <v>40</v>
+      </c>
+      <c r="D331" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B332" s="2">
+        <v>46473</v>
+      </c>
+      <c r="C332">
+        <v>40</v>
+      </c>
+      <c r="D332" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B333" s="2">
+        <v>46474</v>
+      </c>
+      <c r="C333">
+        <v>40</v>
+      </c>
+      <c r="D333" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B334" s="2">
+        <v>46475</v>
+      </c>
+      <c r="C334">
+        <v>40</v>
+      </c>
+      <c r="D334" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B335" s="2">
+        <v>46476</v>
+      </c>
+      <c r="C335">
+        <v>40</v>
+      </c>
+      <c r="D335" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B336" s="2">
+        <v>46477</v>
+      </c>
+      <c r="C336">
+        <v>40</v>
+      </c>
+      <c r="D336" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B337" s="2">
+        <v>46478</v>
+      </c>
+      <c r="C337">
+        <v>40</v>
+      </c>
+      <c r="D337" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B1:D337" xr:uid="{FB4DFB22-8CED-4A0D-BA7D-5E036AC4DBFC}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{58d84362-1b1e-41fa-9f4a-001d35549470}" enabled="1" method="Standard" siteId="{db8e2f82-8a37-4c09-b7de-ed06547b5a20}" contentBits="1" removed="0"/>

</xml_diff>